<commit_message>
J3 : importation, nettoyage et controle qualité
</commit_message>
<xml_diff>
--- a/data/input/clients_test.xlsx
+++ b/data/input/clients_test.xlsx
@@ -39,9 +39,6 @@
     <t>Awa</t>
   </si>
   <si>
-    <t>awa.diop@mail.com</t>
-  </si>
-  <si>
     <t>771234567</t>
   </si>
   <si>
@@ -51,9 +48,6 @@
     <t>moussa</t>
   </si>
   <si>
-    <t>moussa.fall@mail</t>
-  </si>
-  <si>
     <t>770000000</t>
   </si>
   <si>
@@ -63,9 +57,6 @@
     <t>Fatou</t>
   </si>
   <si>
-    <t>Fatou@Mail.COM</t>
-  </si>
-  <si>
     <t>781112223</t>
   </si>
   <si>
@@ -75,9 +66,6 @@
     <t xml:space="preserve">  Cheikh</t>
   </si>
   <si>
-    <t>cheikh.sow@mail.com</t>
-  </si>
-  <si>
     <t>Ba</t>
   </si>
   <si>
@@ -90,20 +78,40 @@
     <t>Omar</t>
   </si>
   <si>
-    <t>omar@@mail.com</t>
-  </si>
-  <si>
     <t>770001111</t>
+  </si>
+  <si>
+    <t>awa.diop@gmail.com</t>
+  </si>
+  <si>
+    <t>moussa.fall@gmail</t>
+  </si>
+  <si>
+    <t>Fatou@GMail.COM</t>
+  </si>
+  <si>
+    <t>cheikh.sow@gmail.com</t>
+  </si>
+  <si>
+    <t>omar@@gmail.com</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -126,13 +134,16 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Lien hypertexte" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -462,89 +473,96 @@
       <c r="B2" t="s">
         <v>5</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D2" t="s">
         <v>6</v>
-      </c>
-      <c r="D2" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" t="s">
         <v>8</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D3" t="s">
         <v>9</v>
-      </c>
-      <c r="C3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D3" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D4" t="s">
         <v>12</v>
-      </c>
-      <c r="B4" t="s">
-        <v>13</v>
-      </c>
-      <c r="C4" t="s">
-        <v>14</v>
-      </c>
-      <c r="D4" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D5" t="s">
         <v>12</v>
-      </c>
-      <c r="B5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" t="s">
-        <v>14</v>
-      </c>
-      <c r="D5" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="B6" t="s">
-        <v>17</v>
-      </c>
-      <c r="C6" t="s">
-        <v>18</v>
+        <v>14</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="B7" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="D7" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B8" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="C8" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D8" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C2" r:id="rId1"/>
+    <hyperlink ref="C3" r:id="rId2"/>
+    <hyperlink ref="C4" r:id="rId3"/>
+    <hyperlink ref="C5" r:id="rId4"/>
+    <hyperlink ref="C6" r:id="rId5"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>